<commit_message>
rename figure for publish
</commit_message>
<xml_diff>
--- a/publishing/accessibility/springer_alt_text_inventory.xlsx
+++ b/publishing/accessibility/springer_alt_text_inventory.xlsx
@@ -686,7 +686,7 @@
       </c>
       <c r="K3" s="8" t="inlineStr">
         <is>
-          <t>docs/images/book_structure_en.png</t>
+          <t>docs/images/Yu-FrontMatter-Fig02-EN.png</t>
         </is>
       </c>
       <c r="L3" s="8" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="K4" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part1/data_engineering_roles_1775830393574.svg</t>
+          <t>docs/images/part1/Yu-Chap01-Fig01.svg</t>
         </is>
       </c>
       <c r="L4" s="8" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="K5" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part1/data_lifecycle_map_1775830407042.svg</t>
+          <t>docs/images/part1/Yu-Chap01-Fig02.svg</t>
         </is>
       </c>
       <c r="L5" s="8" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="K6" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part1/data_quality_hierarchy_1775835516841.svg</t>
+          <t>docs/images/part1/Yu-Chap02-Fig01.svg</t>
         </is>
       </c>
       <c r="L6" s="8" t="inlineStr">
@@ -982,7 +982,7 @@
       </c>
       <c r="K7" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part1/defect_metric_radar_1775835533937.svg</t>
+          <t>docs/images/part1/Yu-Chap02-Fig02.svg</t>
         </is>
       </c>
       <c r="L7" s="8" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part1/data_quality_gates_1775835548587.svg</t>
+          <t>docs/images/part1/Yu-Chap02-Fig03.svg</t>
         </is>
       </c>
       <c r="L8" s="8" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="K9" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part1/ai_data_stack_architecture.svg</t>
+          <t>docs/images/part1/Yu-Chap03-Fig01.svg</t>
         </is>
       </c>
       <c r="L9" s="8" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="K10" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part1/cost_governance_loop.svg</t>
+          <t>docs/images/part1/Yu-Chap03-Fig02.svg</t>
         </is>
       </c>
       <c r="L10" s="8" t="inlineStr">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="K11" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part10/ai_agent_decision_workflow_ch31_01.svg</t>
+          <t>docs/images/part10/Yu-Chap31-Fig01.svg</t>
         </is>
       </c>
       <c r="L11" s="8" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="K12" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part10/ai_agent_decision_workflow_ch31_02.svg</t>
+          <t>docs/images/part10/Yu-Chap31-Fig02.svg</t>
         </is>
       </c>
       <c r="L12" s="8" t="inlineStr">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="K13" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part10/ai_agent_decision_workflow_ch32_01.svg</t>
+          <t>docs/images/part10/Yu-Chap32-Fig01.svg</t>
         </is>
       </c>
       <c r="L13" s="8" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="K14" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part10/ai_agent_decision_workflow_ch32_02.svg</t>
+          <t>docs/images/part10/Yu-Chap32-Fig02.svg</t>
         </is>
       </c>
       <c r="L14" s="8" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="K15" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part10/ai_agent_decision_workflow_ch32_03.svg</t>
+          <t>docs/images/part10/Yu-Chap32-Fig03.svg</t>
         </is>
       </c>
       <c r="L15" s="8" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="K16" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part10/ai_agent_decision_workflow_ch33_01.svg</t>
+          <t>docs/images/part10/Wang-Chap33-Fig01.svg</t>
         </is>
       </c>
       <c r="L16" s="8" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="K17" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part10/ai_agent_decision_workflow_ch33_02.svg</t>
+          <t>docs/images/part10/Wang-Chap33-Fig02.svg</t>
         </is>
       </c>
       <c r="L17" s="8" t="inlineStr">
@@ -1796,7 +1796,7 @@
       </c>
       <c r="K18" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part10/ai_agent_decision_workflow_ch34_01.svg</t>
+          <t>docs/images/part10/Luo-Chap34-Fig01.svg</t>
         </is>
       </c>
       <c r="L18" s="8" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="K19" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part10/ai_agent_decision_workflow_ch34_02.svg</t>
+          <t>docs/images/part10/Luo-Chap34-Fig02.svg</t>
         </is>
       </c>
       <c r="L19" s="8" t="inlineStr">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="K20" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part10/ai_agent_decision_workflow_ch34_03.svg</t>
+          <t>docs/images/part10/Luo-Chap34-Fig03.svg</t>
         </is>
       </c>
       <c r="L20" s="8" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="K21" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part10/ai_agent_decision_workflow_ch35_01.svg</t>
+          <t>docs/images/part10/Luo-Chap35-Fig01.svg</t>
         </is>
       </c>
       <c r="L21" s="8" t="inlineStr">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="K22" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part10/ai_agent_decision_workflow_ch35_02.svg</t>
+          <t>docs/images/part10/Luo-Chap35-Fig02.svg</t>
         </is>
       </c>
       <c r="L22" s="8" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="K23" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part10/ai_agent_decision_workflow_ch35_03.svg</t>
+          <t>docs/images/part10/Luo-Chap35-Fig03.svg</t>
         </is>
       </c>
       <c r="L23" s="8" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="K24" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图36_1_合规左移与治理协同架构图.svg</t>
+          <t>docs/images/part11/Wang-Chap36-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L24" s="8" t="inlineStr">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="K25" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图36_4_数据分级用途和处理动作构成的风险矩阵图.svg</t>
+          <t>docs/images/part11/Wang-Chap36-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L25" s="8" t="inlineStr">
@@ -2388,7 +2388,7 @@
       </c>
       <c r="K26" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图36_5_从数据接入到模型训练的合规门禁流程图.svg</t>
+          <t>docs/images/part11/Wang-Chap36-Fig03-ZH.svg</t>
         </is>
       </c>
       <c r="L26" s="8" t="inlineStr">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="K27" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图36_3_P09隐私规格与策略生成流程图.svg</t>
+          <t>docs/images/part11/Wang-Chap36-Fig04-ZH.svg</t>
         </is>
       </c>
       <c r="L27" s="8" t="inlineStr">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="K28" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图36_2_DPIA与RoPA工程化审批流.svg</t>
+          <t>docs/images/part11/Wang-Chap36-Fig05-ZH.svg</t>
         </is>
       </c>
       <c r="L28" s="8" t="inlineStr">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="K29" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图36_6_审计日志告警事件响应与复盘闭环图.svg</t>
+          <t>docs/images/part11/Wang-Chap36-Fig06-ZH.svg</t>
         </is>
       </c>
       <c r="L29" s="8" t="inlineStr">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="K30" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图36_7_第三方API与大模型调用边界网关图.svg</t>
+          <t>docs/images/part11/Wang-Chap36-Fig07-ZH.svg</t>
         </is>
       </c>
       <c r="L30" s="8" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="K31" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图36_8_用户删除请求的全链路传播与清理示意图.svg</t>
+          <t>docs/images/part11/Wang-Chap36-Fig08-ZH.svg</t>
         </is>
       </c>
       <c r="L31" s="8" t="inlineStr">
@@ -2832,7 +2832,7 @@
       </c>
       <c r="K32" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图37_1_跨机构医疗数据协作中的隐私与合规冲突示意图.svg</t>
+          <t>docs/images/part11/Wang-Chap37-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L32" s="8" t="inlineStr">
@@ -2906,7 +2906,7 @@
       </c>
       <c r="K33" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图37_2_数据可用性与隐私保护的结构性矛盾示意图.svg</t>
+          <t>docs/images/part11/Wang-Chap37-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L33" s="8" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="K34" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图37_3_从数据安全到训练安全的治理重心迁移图.svg</t>
+          <t>docs/images/part11/Wang-Chap37-Fig03-ZH.svg</t>
         </is>
       </c>
       <c r="L34" s="8" t="inlineStr">
@@ -3054,7 +3054,7 @@
       </c>
       <c r="K35" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图37_4_隐私增强技术全景矩阵图.svg</t>
+          <t>docs/images/part11/Wang-Chap37-Fig04-ZH.svg</t>
         </is>
       </c>
       <c r="L35" s="8" t="inlineStr">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="K36" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图37_5_联邦学习基本训练闭环.svg</t>
+          <t>docs/images/part11/Wang-Chap37-Fig05-ZH.svg</t>
         </is>
       </c>
       <c r="L36" s="8" t="inlineStr">
@@ -3202,7 +3202,7 @@
       </c>
       <c r="K37" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图37_6_DPSGD训练流程示意图.svg</t>
+          <t>docs/images/part11/Wang-Chap37-Fig06-ZH.svg</t>
         </is>
       </c>
       <c r="L37" s="8" t="inlineStr">
@@ -3276,7 +3276,7 @@
       </c>
       <c r="K38" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图37_7_联邦训练中的通信成本分解图.svg</t>
+          <t>docs/images/part11/Wang-Chap37-Fig07-ZH.svg</t>
         </is>
       </c>
       <c r="L38" s="8" t="inlineStr">
@@ -3350,7 +3350,7 @@
       </c>
       <c r="K39" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图37_8_横向联邦与纵向联邦对比示意图.svg</t>
+          <t>docs/images/part11/Wang-Chap37-Fig08-ZH.svg</t>
         </is>
       </c>
       <c r="L39" s="8" t="inlineStr">
@@ -3424,7 +3424,7 @@
       </c>
       <c r="K40" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图37_9_梯度反演攻击示意图.svg</t>
+          <t>docs/images/part11/Wang-Chap37-Fig09-ZH.svg</t>
         </is>
       </c>
       <c r="L40" s="8" t="inlineStr">
@@ -3498,7 +3498,7 @@
       </c>
       <c r="K41" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图37_10_联邦系统整体架构图.svg</t>
+          <t>docs/images/part11/Wang-Chap37-Fig10-ZH.svg</t>
         </is>
       </c>
       <c r="L41" s="8" t="inlineStr">
@@ -3572,7 +3572,7 @@
       </c>
       <c r="K42" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图37_11_合规治理隐私流水线联邦训练与应用能力闭环图.svg</t>
+          <t>docs/images/part11/Wang-Chap37-Fig11-ZH.svg</t>
         </is>
       </c>
       <c r="L42" s="8" t="inlineStr">
@@ -3646,7 +3646,7 @@
       </c>
       <c r="K43" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part11/图37_12_医疗与金融场景的隐私技术路线对比图.svg</t>
+          <t>docs/images/part11/Wang-Chap37-Fig12-ZH.svg</t>
         </is>
       </c>
       <c r="L43" s="8" t="inlineStr">
@@ -3720,7 +3720,7 @@
       </c>
       <c r="K44" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch38_01_fineweb_minhash_pii_flow_en.svg</t>
+          <t>docs/images/part12/Mu-Chap38-Fig01-EN.svg</t>
         </is>
       </c>
       <c r="L44" s="8" t="inlineStr">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="K45" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch38_02_fineweb_ablation_loop_en.svg</t>
+          <t>docs/images/part12/Mu-Chap38-Fig02-EN.svg</t>
         </is>
       </c>
       <c r="L45" s="8" t="inlineStr">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="K46" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch38_03_dolma_evidence_chain_en.svg</t>
+          <t>docs/images/part12/Mu-Chap38-Fig03-EN.svg</t>
         </is>
       </c>
       <c r="L46" s="8" t="inlineStr">
@@ -3942,7 +3942,7 @@
       </c>
       <c r="K47" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch38_04_dolma_source_mix_diagnosis_en.svg</t>
+          <t>docs/images/part12/Mu-Chap38-Fig04-EN.svg</t>
         </is>
       </c>
       <c r="L47" s="8" t="inlineStr">
@@ -4016,7 +4016,7 @@
       </c>
       <c r="K48" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch39_01_laion_multichannel_schema_en.svg</t>
+          <t>docs/images/part12/Mu-Chap39-Fig01-EN.svg</t>
         </is>
       </c>
       <c r="L48" s="8" t="inlineStr">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="K49" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch39_02_laion_quality_datacomp_loop_en.svg</t>
+          <t>docs/images/part12/Mu-Chap39-Fig02-EN.svg</t>
         </is>
       </c>
       <c r="L49" s="8" t="inlineStr">
@@ -4193,7 +4193,7 @@
       </c>
       <c r="K50" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch40_01_schema_decomposition_en.png</t>
+          <t>docs/images/part12/Liu-Chap40-Fig01-EN.png</t>
         </is>
       </c>
       <c r="L50" s="8" t="inlineStr">
@@ -4271,7 +4271,7 @@
       </c>
       <c r="K51" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch40_02_dataset_construction_pipeline_en.png</t>
+          <t>docs/images/part12/Liu-Chap40-Fig02-EN.png</t>
         </is>
       </c>
       <c r="L51" s="8" t="inlineStr">
@@ -4349,7 +4349,7 @@
       </c>
       <c r="K52" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch40_03_structural_consistency_validation_en.png</t>
+          <t>docs/images/part12/Liu-Chap40-Fig03-EN.png</t>
         </is>
       </c>
       <c r="L52" s="8" t="inlineStr">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="K53" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch40_04_supervision_schema_en.png</t>
+          <t>docs/images/part12/Liu-Chap40-Fig04-EN.png</t>
         </is>
       </c>
       <c r="L53" s="8" t="inlineStr">
@@ -4505,7 +4505,7 @@
       </c>
       <c r="K54" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch40_05_stb_pipeline_en.png</t>
+          <t>docs/images/part12/Liu-Chap40-Fig05-EN.png</t>
         </is>
       </c>
       <c r="L54" s="8" t="inlineStr">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="K55" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch40_06_mask_stress_flow_en.png</t>
+          <t>docs/images/part12/Liu-Chap40-Fig06-EN.png</t>
         </is>
       </c>
       <c r="L55" s="8" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="K56" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch41_01_domain_distribution_en.png</t>
+          <t>docs/images/part12/Xu-Chap41-Fig01-EN.png</t>
         </is>
       </c>
       <c r="L56" s="8" t="inlineStr">
@@ -4735,7 +4735,7 @@
       </c>
       <c r="K57" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch41_02_chart_type_distribution_en.png</t>
+          <t>docs/images/part12/Xu-Chap41-Fig02-EN.png</t>
         </is>
       </c>
       <c r="L57" s="8" t="inlineStr">
@@ -4809,7 +4809,7 @@
       </c>
       <c r="K58" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch41_03_question_type_distribution_en.png</t>
+          <t>docs/images/part12/Xu-Chap41-Fig03-EN.png</t>
         </is>
       </c>
       <c r="L58" s="8" t="inlineStr">
@@ -4881,7 +4881,7 @@
       </c>
       <c r="K59" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch41_04_shark_attack_infographic_1.jpg</t>
+          <t>docs/images/part12/Xu-Chap41-Fig04-Alt02.jpg</t>
         </is>
       </c>
       <c r="L59" s="8" t="inlineStr">
@@ -4953,7 +4953,7 @@
       </c>
       <c r="K60" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch41_04_shark_attack_infographic_2.jpg</t>
+          <t>docs/images/part12/Xu-Chap41-Fig04-Alt03.jpg</t>
         </is>
       </c>
       <c r="L60" s="8" t="inlineStr">
@@ -5021,7 +5021,7 @@
       </c>
       <c r="K61" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch41_04_shark_attack_infographic_3.jpg</t>
+          <t>docs/images/part12/Xu-Chap41-Fig04-Alt04.jpg</t>
         </is>
       </c>
       <c r="L61" s="8" t="inlineStr">
@@ -5089,7 +5089,7 @@
       </c>
       <c r="K62" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch41_04_shark_attack_infographic_4.jpg</t>
+          <t>docs/images/part12/Xu-Chap41-Fig04-Alt05.jpg</t>
         </is>
       </c>
       <c r="L62" s="8" t="inlineStr">
@@ -5159,7 +5159,7 @@
       </c>
       <c r="K63" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch41_05_multichart_dataset_pipeline_en.png</t>
+          <t>docs/images/part12/Xu-Chap41-Fig05-EN.png</t>
         </is>
       </c>
       <c r="L63" s="8" t="inlineStr">
@@ -5233,7 +5233,7 @@
       </c>
       <c r="K64" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch41_06_medimage_tool_vqa_pipeline_en.svg</t>
+          <t>docs/images/part12/Xu-Chap41-Fig06-EN.svg</t>
         </is>
       </c>
       <c r="L64" s="8" t="inlineStr">
@@ -5321,7 +5321,7 @@
       </c>
       <c r="K65" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch41_07_tool_trajectory_structure_en.svg</t>
+          <t>docs/images/part12/Xu-Chap41-Fig07-EN.svg</t>
         </is>
       </c>
       <c r="L65" s="8" t="inlineStr">
@@ -5409,7 +5409,7 @@
       </c>
       <c r="K66" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch41_08_sft_schema_real_bbox_example_en.svg</t>
+          <t>docs/images/part12/Xu-Chap41-Fig08-EN.svg</t>
         </is>
       </c>
       <c r="L66" s="8" t="inlineStr">
@@ -5487,7 +5487,7 @@
       </c>
       <c r="K67" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch41_09_quality_review_gate_en.svg</t>
+          <t>docs/images/part12/Xu-Chap41-Fig09-EN.svg</t>
         </is>
       </c>
       <c r="L67" s="8" t="inlineStr">
@@ -5565,7 +5565,7 @@
       </c>
       <c r="K68" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch42_01_dual_channel_schema_en.svg</t>
+          <t>docs/images/part12/Chen-Chap42-Fig01-EN.svg</t>
         </is>
       </c>
       <c r="L68" s="8" t="inlineStr">
@@ -5639,7 +5639,7 @@
       </c>
       <c r="K69" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch42_02_voice_style_data_pipeline_en.svg</t>
+          <t>docs/images/part12/Chen-Chap42-Fig02-EN.svg</t>
         </is>
       </c>
       <c r="L69" s="8" t="inlineStr">
@@ -5713,7 +5713,7 @@
       </c>
       <c r="K70" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch42_03_quality_loop_en.svg</t>
+          <t>docs/images/part12/Chen-Chap42-Fig03-EN.svg</t>
         </is>
       </c>
       <c r="L70" s="8" t="inlineStr">
@@ -5787,7 +5787,7 @@
       </c>
       <c r="K71" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch43_01_latent_switch_pipeline.svg</t>
+          <t>docs/images/part12/Li-Chap43-Fig01.svg</t>
         </is>
       </c>
       <c r="L71" s="8" t="inlineStr">
@@ -5865,7 +5865,7 @@
       </c>
       <c r="K72" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch43_02_dataset_composition.png</t>
+          <t>docs/images/part12/Li-Chap43-Fig02.png</t>
         </is>
       </c>
       <c r="L72" s="8" t="inlineStr">
@@ -5943,7 +5943,7 @@
       </c>
       <c r="K73" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch43_03_cot_latent_comparison.svg</t>
+          <t>docs/images/part12/Li-Chap43-Fig03.svg</t>
         </is>
       </c>
       <c r="L73" s="8" t="inlineStr">
@@ -6021,7 +6021,7 @@
       </c>
       <c r="K74" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch43_04_token_compression_distribution.png</t>
+          <t>docs/images/part12/Li-Chap43-Fig04.png</t>
         </is>
       </c>
       <c r="L74" s="8" t="inlineStr">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="K75" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part12/ch43_05_supervision_mask.svg</t>
+          <t>docs/images/part12/Li-Chap43-Fig05.svg</t>
         </is>
       </c>
       <c r="L75" s="8" t="inlineStr">
@@ -6177,7 +6177,7 @@
       </c>
       <c r="K76" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch44_01_data_recipe_funnel_en.svg</t>
+          <t>docs/images/part13/Wang-Chap44-Fig01-EN.svg</t>
         </is>
       </c>
       <c r="L76" s="8" t="inlineStr">
@@ -6255,7 +6255,7 @@
       </c>
       <c r="K77" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch44_02_data_transparency_spectrum_en.svg</t>
+          <t>docs/images/part13/Wang-Chap44-Fig02-EN.svg</t>
         </is>
       </c>
       <c r="L77" s="8" t="inlineStr">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="K78" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch44_03_pretrain_data_source_map.png</t>
+          <t>docs/images/part13/Wang-Chap44-Fig03.png</t>
         </is>
       </c>
       <c r="L78" s="8" t="inlineStr">
@@ -6411,7 +6411,7 @@
       </c>
       <c r="K79" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch44_04_models_pie_chart_en.svg</t>
+          <t>docs/images/part13/Wang-Chap44-Fig04-EN.svg</t>
         </is>
       </c>
       <c r="L79" s="8" t="inlineStr">
@@ -6489,7 +6489,7 @@
       </c>
       <c r="K80" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch44_05_llama3_annealing_schedule_en.svg</t>
+          <t>docs/images/part13/Wang-Chap44-Fig05-EN.svg</t>
         </is>
       </c>
       <c r="L80" s="8" t="inlineStr">
@@ -6567,7 +6567,7 @@
       </c>
       <c r="K81" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch45_01_posttrain_three_stage_pipeline.svg</t>
+          <t>docs/images/part13/Wang-Chap45-Fig01.svg</t>
         </is>
       </c>
       <c r="L81" s="8" t="inlineStr">
@@ -6645,7 +6645,7 @@
       </c>
       <c r="K82" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch45_02_sft_synthesis_pipelines.svg</t>
+          <t>docs/images/part13/Wang-Chap45-Fig02.svg</t>
         </is>
       </c>
       <c r="L82" s="8" t="inlineStr">
@@ -6723,7 +6723,7 @@
       </c>
       <c r="K83" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch45_03_tulu3_posttrain_flow.svg</t>
+          <t>docs/images/part13/Wang-Chap45-Fig03.svg</t>
         </is>
       </c>
       <c r="L83" s="8" t="inlineStr">
@@ -6801,7 +6801,7 @@
       </c>
       <c r="K84" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch46_01_r1_reasoning_flywheel.svg</t>
+          <t>docs/images/part13/Xu-Chap46-Fig01.svg</t>
         </is>
       </c>
       <c r="L84" s="8" t="inlineStr">
@@ -6879,7 +6879,7 @@
       </c>
       <c r="K85" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch46_02_reward_verifier_architecture.svg</t>
+          <t>docs/images/part13/Xu-Chap46-Fig02.svg</t>
         </is>
       </c>
       <c r="L85" s="8" t="inlineStr">
@@ -6957,7 +6957,7 @@
       </c>
       <c r="K86" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch46_03_long_cot_trace_patterns.svg</t>
+          <t>docs/images/part13/Xu-Chap46-Fig03.svg</t>
         </is>
       </c>
       <c r="L86" s="8" t="inlineStr">
@@ -7035,7 +7035,7 @@
       </c>
       <c r="K87" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch47_01_multimodal_data_panorama.png</t>
+          <t>docs/images/part13/Cao-Chap47-Fig01.png</t>
         </is>
       </c>
       <c r="L87" s="8" t="inlineStr">
@@ -7113,7 +7113,7 @@
       </c>
       <c r="K88" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch47_02_vlm_three_stages_en.svg</t>
+          <t>docs/images/part13/Cao-Chap47-Fig02-EN.svg</t>
         </is>
       </c>
       <c r="L88" s="8" t="inlineStr">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="K89" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch47_03_resolution_handling_en.svg</t>
+          <t>docs/images/part13/Cao-Chap47-Fig03-EN.svg</t>
         </is>
       </c>
       <c r="L89" s="8" t="inlineStr">
@@ -7269,7 +7269,7 @@
       </c>
       <c r="K90" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch47_04_instruction_synthesis_en.svg</t>
+          <t>docs/images/part13/Cao-Chap47-Fig04-EN.svg</t>
         </is>
       </c>
       <c r="L90" s="8" t="inlineStr">
@@ -7347,7 +7347,7 @@
       </c>
       <c r="K91" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch48_01_t2i_data_pipeline.svg</t>
+          <t>docs/images/part13/Zhang-Chap48-Fig01.svg</t>
         </is>
       </c>
       <c r="L91" s="8" t="inlineStr">
@@ -7421,7 +7421,7 @@
       </c>
       <c r="K92" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch48_02_t2v_data_pipeline.svg</t>
+          <t>docs/images/part13/Zhang-Chap48-Fig02.svg</t>
         </is>
       </c>
       <c r="L92" s="8" t="inlineStr">
@@ -7495,7 +7495,7 @@
       </c>
       <c r="K93" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part13/ch48_03_multistage_filtering_architecture.svg</t>
+          <t>docs/images/part13/Zhang-Chap48-Fig03.svg</t>
         </is>
       </c>
       <c r="L93" s="8" t="inlineStr">
@@ -7571,7 +7571,7 @@
       </c>
       <c r="K94" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p01/p01_01_mini_c4_pipeline_overview.svg</t>
+          <t>docs/images/part14/p01/Xu-Project01-Fig01.svg</t>
         </is>
       </c>
       <c r="L94" s="8" t="inlineStr">
@@ -7651,7 +7651,7 @@
       </c>
       <c r="K95" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p01/p01_02_warc_to_text.svg</t>
+          <t>docs/images/part14/p01/Xu-Project01-Fig02.svg</t>
         </is>
       </c>
       <c r="L95" s="8" t="inlineStr">
@@ -7731,7 +7731,7 @@
       </c>
       <c r="K96" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p01/p01_03_cleaning_rules.svg</t>
+          <t>docs/images/part14/p01/Xu-Project01-Fig03.svg</t>
         </is>
       </c>
       <c r="L96" s="8" t="inlineStr">
@@ -7807,7 +7807,7 @@
       </c>
       <c r="K97" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p01/p01_04_dedup_minhash_lsh.svg</t>
+          <t>docs/images/part14/p01/Xu-Project01-Fig04.svg</t>
         </is>
       </c>
       <c r="L97" s="8" t="inlineStr">
@@ -7887,7 +7887,7 @@
       </c>
       <c r="K98" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p01/p01_05_language_split.svg</t>
+          <t>docs/images/part14/p01/Xu-Project01-Fig05.svg</t>
         </is>
       </c>
       <c r="L98" s="8" t="inlineStr">
@@ -7967,7 +7967,7 @@
       </c>
       <c r="K99" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p01/p01_06_quality_filter.svg</t>
+          <t>docs/images/part14/p01/Xu-Project01-Fig06.svg</t>
         </is>
       </c>
       <c r="L99" s="8" t="inlineStr">
@@ -8047,7 +8047,7 @@
       </c>
       <c r="K100" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p01/p01_07_three_iterations.svg</t>
+          <t>docs/images/part14/p01/Xu-Project01-Fig07.svg</t>
         </is>
       </c>
       <c r="L100" s="8" t="inlineStr">
@@ -8127,7 +8127,7 @@
       </c>
       <c r="K101" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p01/p01_08_funnel.svg</t>
+          <t>docs/images/part14/p01/Xu-Project01-Fig08.svg</t>
         </is>
       </c>
       <c r="L101" s="8" t="inlineStr">
@@ -8207,7 +8207,7 @@
       </c>
       <c r="K102" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p01/p01_09_cost_breakdown.svg</t>
+          <t>docs/images/part14/p01/Xu-Project01-Fig09.svg</t>
         </is>
       </c>
       <c r="L102" s="8" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="K103" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p01/p01_10_validation_loop.svg</t>
+          <t>docs/images/part14/p01/Xu-Project01-Fig10.svg</t>
         </is>
       </c>
       <c r="L103" s="8" t="inlineStr">
@@ -8367,7 +8367,7 @@
       </c>
       <c r="K104" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p01/p01_11_methodology_summary.svg</t>
+          <t>docs/images/part14/p01/Xu-Project01-Fig11.svg</t>
         </is>
       </c>
       <c r="L104" s="8" t="inlineStr">
@@ -8443,7 +8443,7 @@
       </c>
       <c r="K105" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_01_legal_sft_factory_overview.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig01.svg</t>
         </is>
       </c>
       <c r="L105" s="8" t="inlineStr">
@@ -8523,7 +8523,7 @@
       </c>
       <c r="K106" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_02_roles_and_responsibilities.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig02.svg</t>
         </is>
       </c>
       <c r="L106" s="8" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="K107" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_03_pdf_cleaning_pipeline.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig03.svg</t>
         </is>
       </c>
       <c r="L107" s="8" t="inlineStr">
@@ -8679,7 +8679,7 @@
       </c>
       <c r="K108" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_04_cleaning_examples.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig04.svg</t>
         </is>
       </c>
       <c r="L108" s="8" t="inlineStr">
@@ -8755,7 +8755,7 @@
       </c>
       <c r="K109" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_05_seed_schema.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig05.svg</t>
         </is>
       </c>
       <c r="L109" s="8" t="inlineStr">
@@ -8835,7 +8835,7 @@
       </c>
       <c r="K110" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_06_task_taxonomy.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig06.svg</t>
         </is>
       </c>
       <c r="L110" s="8" t="inlineStr">
@@ -8911,7 +8911,7 @@
       </c>
       <c r="K111" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_07_task_vs_domain_distribution.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig07.svg</t>
         </is>
       </c>
       <c r="L111" s="8" t="inlineStr">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="K112" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_08_weighted_task_sampling.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig08.svg</t>
         </is>
       </c>
       <c r="L112" s="8" t="inlineStr">
@@ -9071,7 +9071,7 @@
       </c>
       <c r="K113" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_09_cot_structure.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig09.svg</t>
         </is>
       </c>
       <c r="L113" s="8" t="inlineStr">
@@ -9147,7 +9147,7 @@
       </c>
       <c r="K114" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_10_preference_and_review.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig10.svg</t>
         </is>
       </c>
       <c r="L114" s="8" t="inlineStr">
@@ -9227,7 +9227,7 @@
       </c>
       <c r="K115" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_11_risk_refusal_flow.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig11.svg</t>
         </is>
       </c>
       <c r="L115" s="8" t="inlineStr">
@@ -9307,7 +9307,7 @@
       </c>
       <c r="K116" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_12_qa_loop.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig12.svg</t>
         </is>
       </c>
       <c r="L116" s="8" t="inlineStr">
@@ -9387,7 +9387,7 @@
       </c>
       <c r="K117" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_13_qa_decision_table.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig13.svg</t>
         </is>
       </c>
       <c r="L117" s="8" t="inlineStr">
@@ -9467,7 +9467,7 @@
       </c>
       <c r="K118" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_14_human_in_the_loop.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig14.svg</t>
         </is>
       </c>
       <c r="L118" s="8" t="inlineStr">
@@ -9547,7 +9547,7 @@
       </c>
       <c r="K119" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_15_training_artifacts.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig15.svg</t>
         </is>
       </c>
       <c r="L119" s="8" t="inlineStr">
@@ -9623,7 +9623,7 @@
       </c>
       <c r="K120" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_16_metrics_dashboard.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig16.svg</t>
         </is>
       </c>
       <c r="L120" s="8" t="inlineStr">
@@ -9703,7 +9703,7 @@
       </c>
       <c r="K121" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_17_eval_sampling_protocol.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig17.svg</t>
         </is>
       </c>
       <c r="L121" s="8" t="inlineStr">
@@ -9783,7 +9783,7 @@
       </c>
       <c r="K122" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_18_version_timeline.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig18.svg</t>
         </is>
       </c>
       <c r="L122" s="8" t="inlineStr">
@@ -9863,7 +9863,7 @@
       </c>
       <c r="K123" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_19_validation_chain.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig19.svg</t>
         </is>
       </c>
       <c r="L123" s="8" t="inlineStr">
@@ -9943,7 +9943,7 @@
       </c>
       <c r="K124" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p02/p02_20_cross_domain_transfer.svg</t>
+          <t>docs/images/part14/p02/Xu-Project02-Fig20.svg</t>
         </is>
       </c>
       <c r="L124" s="8" t="inlineStr">
@@ -10019,7 +10019,7 @@
       </c>
       <c r="K125" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p03/p03_01_llava_factory_overview.svg</t>
+          <t>docs/images/part14/p03/Yu-Project03-Fig01.svg</t>
         </is>
       </c>
       <c r="L125" s="8" t="inlineStr">
@@ -10099,7 +10099,7 @@
       </c>
       <c r="K126" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p03/p03_02_roles_and_responsibilities.svg</t>
+          <t>docs/images/part14/p03/Yu-Project03-Fig02.svg</t>
         </is>
       </c>
       <c r="L126" s="8" t="inlineStr">
@@ -10175,7 +10175,7 @@
       </c>
       <c r="K127" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p03/p03_03_asset_layers.svg</t>
+          <t>docs/images/part14/p03/Yu-Project03-Fig03.svg</t>
         </is>
       </c>
       <c r="L127" s="8" t="inlineStr">
@@ -10255,7 +10255,7 @@
       </c>
       <c r="K128" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p03/p03_04_document_tasks.svg</t>
+          <t>docs/images/part14/p03/Yu-Project03-Fig04.svg</t>
         </is>
       </c>
       <c r="L128" s="8" t="inlineStr">
@@ -10331,7 +10331,7 @@
       </c>
       <c r="K129" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p03/p03_05_bbox_alignment.svg</t>
+          <t>docs/images/part14/p03/Yu-Project03-Fig05.svg</t>
         </is>
       </c>
       <c r="L129" s="8" t="inlineStr">
@@ -10411,7 +10411,7 @@
       </c>
       <c r="K130" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p03/p03_06_quality_loop.svg</t>
+          <t>docs/images/part14/p03/Yu-Project03-Fig06.svg</t>
         </is>
       </c>
       <c r="L130" s="8" t="inlineStr">
@@ -10491,7 +10491,7 @@
       </c>
       <c r="K131" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p03/p03_07_failure_attribution.svg</t>
+          <t>docs/images/part14/p03/Yu-Project03-Fig07.svg</t>
         </is>
       </c>
       <c r="L131" s="8" t="inlineStr">
@@ -10571,7 +10571,7 @@
       </c>
       <c r="K132" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p03/p03_08_validation_loop.svg</t>
+          <t>docs/images/part14/p03/Yu-Project03-Fig08.svg</t>
         </is>
       </c>
       <c r="L132" s="8" t="inlineStr">
@@ -10651,7 +10651,7 @@
       </c>
       <c r="K133" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p04/p04_01_project_positioning.svg</t>
+          <t>docs/images/part14/p04/Xu-Project04-Fig01.svg</t>
         </is>
       </c>
       <c r="L133" s="8" t="inlineStr">
@@ -10727,7 +10727,7 @@
       </c>
       <c r="K134" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p04/p04_02_goals_and_scope.svg</t>
+          <t>docs/images/part14/p04/Xu-Project04-Fig02.svg</t>
         </is>
       </c>
       <c r="L134" s="8" t="inlineStr">
@@ -10803,7 +10803,7 @@
       </c>
       <c r="K135" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p04/p04_03_pipeline_overview.svg</t>
+          <t>docs/images/part14/p04/Xu-Project04-Fig03.svg</t>
         </is>
       </c>
       <c r="L135" s="8" t="inlineStr">
@@ -10883,7 +10883,7 @@
       </c>
       <c r="K136" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p04/p04_04_roles_and_responsibilities.svg</t>
+          <t>docs/images/part14/p04/Xu-Project04-Fig04.svg</t>
         </is>
       </c>
       <c r="L136" s="8" t="inlineStr">
@@ -10959,7 +10959,7 @@
       </c>
       <c r="K137" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p04/p04_05_seed_to_plan.svg</t>
+          <t>docs/images/part14/p04/Xu-Project04-Fig05.svg</t>
         </is>
       </c>
       <c r="L137" s="8" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="K138" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p04/p04_06_evol_path.svg</t>
+          <t>docs/images/part14/p04/Xu-Project04-Fig06.svg</t>
         </is>
       </c>
       <c r="L138" s="8" t="inlineStr">
@@ -11119,7 +11119,7 @@
       </c>
       <c r="K139" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p04/p04_07_cot_vs_pot.svg</t>
+          <t>docs/images/part14/p04/Xu-Project04-Fig07.svg</t>
         </is>
       </c>
       <c r="L139" s="8" t="inlineStr">
@@ -11195,7 +11195,7 @@
       </c>
       <c r="K140" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p04/p04_08_generation_chain.svg</t>
+          <t>docs/images/part14/p04/Xu-Project04-Fig08.svg</t>
         </is>
       </c>
       <c r="L140" s="8" t="inlineStr">
@@ -11275,7 +11275,7 @@
       </c>
       <c r="K141" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p04/p04_09_sandbox_validation.svg</t>
+          <t>docs/images/part14/p04/Xu-Project04-Fig09.svg</t>
         </is>
       </c>
       <c r="L141" s="8" t="inlineStr">
@@ -11355,7 +11355,7 @@
       </c>
       <c r="K142" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p04/p04_10_packaging_outputs.svg</t>
+          <t>docs/images/part14/p04/Xu-Project04-Fig10.svg</t>
         </is>
       </c>
       <c r="L142" s="8" t="inlineStr">
@@ -11435,7 +11435,7 @@
       </c>
       <c r="K143" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p04/p04_11_training_interface.svg</t>
+          <t>docs/images/part14/p04/Xu-Project04-Fig11.svg</t>
         </is>
       </c>
       <c r="L143" s="8" t="inlineStr">
@@ -11515,7 +11515,7 @@
       </c>
       <c r="K144" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p05/p05_01_overall_architecture.svg</t>
+          <t>docs/images/part14/p05/Cao-Project05-Fig01.svg</t>
         </is>
       </c>
       <c r="L144" s="8" t="inlineStr">
@@ -11595,7 +11595,7 @@
       </c>
       <c r="K145" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p05/p05_02_vision_vs_ocr.svg</t>
+          <t>docs/images/part14/p05/Cao-Project05-Fig02.svg</t>
         </is>
       </c>
       <c r="L145" s="8" t="inlineStr">
@@ -11675,7 +11675,7 @@
       </c>
       <c r="K146" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p05/p05_03_page_assets.svg</t>
+          <t>docs/images/part14/p05/Cao-Project05-Fig03.svg</t>
         </is>
       </c>
       <c r="L146" s="8" t="inlineStr">
@@ -11755,7 +11755,7 @@
       </c>
       <c r="K147" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p05/p05_04_indexing_pipeline.svg</t>
+          <t>docs/images/part14/p05/Cao-Project05-Fig04.svg</t>
         </is>
       </c>
       <c r="L147" s="8" t="inlineStr">
@@ -11835,7 +11835,7 @@
       </c>
       <c r="K148" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p05/p05_05_topk_filtering.svg</t>
+          <t>docs/images/part14/p05/Cao-Project05-Fig05.svg</t>
         </is>
       </c>
       <c r="L148" s="8" t="inlineStr">
@@ -11915,7 +11915,7 @@
       </c>
       <c r="K149" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p05/p05_06_multi_image_prompting.svg</t>
+          <t>docs/images/part14/p05/Cao-Project05-Fig06.svg</t>
         </is>
       </c>
       <c r="L149" s="8" t="inlineStr">
@@ -11995,7 +11995,7 @@
       </c>
       <c r="K150" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p05/p05_07_eval_framework.svg</t>
+          <t>docs/images/part14/p05/Cao-Project05-Fig07.svg</t>
         </is>
       </c>
       <c r="L150" s="8" t="inlineStr">
@@ -12075,7 +12075,7 @@
       </c>
       <c r="K151" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p05/p05_08_optimization_roadmap.svg</t>
+          <t>docs/images/part14/p05/Cao-Project05-Fig08.svg</t>
         </is>
       </c>
       <c r="L151" s="8" t="inlineStr">
@@ -12155,7 +12155,7 @@
       </c>
       <c r="K152" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p05/p05_09_hybrid_rag.svg</t>
+          <t>docs/images/part14/p05/Cao-Project05-Fig09.svg</t>
         </is>
       </c>
       <c r="L152" s="8" t="inlineStr">
@@ -12235,7 +12235,7 @@
       </c>
       <c r="K153" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p06/p06_01_prm_factory_overview.svg</t>
+          <t>docs/images/part14/p06/Wang-Project06-Fig01.svg</t>
         </is>
       </c>
       <c r="L153" s="8" t="inlineStr">
@@ -12315,7 +12315,7 @@
       </c>
       <c r="K154" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p06/p06_02_step_validation_loop.svg</t>
+          <t>docs/images/part14/p06/Wang-Project06-Fig02.svg</t>
         </is>
       </c>
       <c r="L154" s="8" t="inlineStr">
@@ -12395,7 +12395,7 @@
       </c>
       <c r="K155" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p06/p06_03_task_sampling.svg</t>
+          <t>docs/images/part14/p06/Wang-Project06-Fig03.svg</t>
         </is>
       </c>
       <c r="L155" s="8" t="inlineStr">
@@ -12475,7 +12475,7 @@
       </c>
       <c r="K156" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p06/p06_04_trace_types.svg</t>
+          <t>docs/images/part14/p06/Wang-Project06-Fig04.svg</t>
         </is>
       </c>
       <c r="L156" s="8" t="inlineStr">
@@ -12551,7 +12551,7 @@
       </c>
       <c r="K157" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p06/p06_05_step_schema.svg</t>
+          <t>docs/images/part14/p06/Wang-Project06-Fig05.svg</t>
         </is>
       </c>
       <c r="L157" s="8" t="inlineStr">
@@ -12631,7 +12631,7 @@
       </c>
       <c r="K158" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p06/p06_06_validation_pipeline.svg</t>
+          <t>docs/images/part14/p06/Wang-Project06-Fig06.svg</t>
         </is>
       </c>
       <c r="L158" s="8" t="inlineStr">
@@ -12711,7 +12711,7 @@
       </c>
       <c r="K159" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p06/p06_07_step_labels.svg</t>
+          <t>docs/images/part14/p06/Wang-Project06-Fig07.svg</t>
         </is>
       </c>
       <c r="L159" s="8" t="inlineStr">
@@ -12787,7 +12787,7 @@
       </c>
       <c r="K160" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p06/p06_08_training_interface.svg</t>
+          <t>docs/images/part14/p06/Wang-Project06-Fig08.svg</t>
         </is>
       </c>
       <c r="L160" s="8" t="inlineStr">
@@ -12867,7 +12867,7 @@
       </c>
       <c r="K161" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p06/p06_09_validation_metrics.svg</t>
+          <t>docs/images/part14/p06/Wang-Project06-Fig09.svg</t>
         </is>
       </c>
       <c r="L161" s="8" t="inlineStr">
@@ -12947,7 +12947,7 @@
       </c>
       <c r="K162" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p06/p06_10_noise_sources.svg</t>
+          <t>docs/images/part14/p06/Wang-Project06-Fig10.svg</t>
         </is>
       </c>
       <c r="L162" s="8" t="inlineStr">
@@ -13027,7 +13027,7 @@
       </c>
       <c r="K163" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p07/p07_01_agent_tooluse_factory_overview.svg</t>
+          <t>docs/images/part14/p07/Yu-Project07-Fig01.svg</t>
         </is>
       </c>
       <c r="L163" s="8" t="inlineStr">
@@ -13107,7 +13107,7 @@
       </c>
       <c r="K164" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p07/p07_02_three_layer_architecture.svg</t>
+          <t>docs/images/part14/p07/Yu-Project07-Fig02.svg</t>
         </is>
       </c>
       <c r="L164" s="8" t="inlineStr">
@@ -13187,7 +13187,7 @@
       </c>
       <c r="K165" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p07/p07_03_roles_and_responsibilities.svg</t>
+          <t>docs/images/part14/p07/Yu-Project07-Fig03.svg</t>
         </is>
       </c>
       <c r="L165" s="8" t="inlineStr">
@@ -13263,7 +13263,7 @@
       </c>
       <c r="K166" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p07/p07_04_tool_schema_structure.svg</t>
+          <t>docs/images/part14/p07/Yu-Project07-Fig04.svg</t>
         </is>
       </c>
       <c r="L166" s="8" t="inlineStr">
@@ -13343,7 +13343,7 @@
       </c>
       <c r="K167" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p07/p07_05_task_specs_and_templates.svg</t>
+          <t>docs/images/part14/p07/Yu-Project07-Fig05.svg</t>
         </is>
       </c>
       <c r="L167" s="8" t="inlineStr">
@@ -13423,7 +13423,7 @@
       </c>
       <c r="K168" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p07/p07_06_trajectory_taxonomy.svg</t>
+          <t>docs/images/part14/p07/Yu-Project07-Fig06.svg</t>
         </is>
       </c>
       <c r="L168" s="8" t="inlineStr">
@@ -13503,7 +13503,7 @@
       </c>
       <c r="K169" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p07/p07_07_simulated_env_loop.svg</t>
+          <t>docs/images/part14/p07/Yu-Project07-Fig07.svg</t>
         </is>
       </c>
       <c r="L169" s="8" t="inlineStr">
@@ -13583,7 +13583,7 @@
       </c>
       <c r="K170" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p07/p07_08_pipeline_steps.svg</t>
+          <t>docs/images/part14/p07/Yu-Project07-Fig08.svg</t>
         </is>
       </c>
       <c r="L170" s="8" t="inlineStr">
@@ -13663,7 +13663,7 @@
       </c>
       <c r="K171" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p07/p07_09_recovery_flow.svg</t>
+          <t>docs/images/part14/p07/Yu-Project07-Fig09.svg</t>
         </is>
       </c>
       <c r="L171" s="8" t="inlineStr">
@@ -13743,7 +13743,7 @@
       </c>
       <c r="K172" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p07/p07_10_memory_trajectory.svg</t>
+          <t>docs/images/part14/p07/Yu-Project07-Fig10.svg</t>
         </is>
       </c>
       <c r="L172" s="8" t="inlineStr">
@@ -13823,7 +13823,7 @@
       </c>
       <c r="K173" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p07/p07_11_unsafe_block.svg</t>
+          <t>docs/images/part14/p07/Yu-Project07-Fig11.svg</t>
         </is>
       </c>
       <c r="L173" s="8" t="inlineStr">
@@ -13903,7 +13903,7 @@
       </c>
       <c r="K174" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p07/p07_12_dataset_repacking.svg</t>
+          <t>docs/images/part14/p07/Yu-Project07-Fig12.svg</t>
         </is>
       </c>
       <c r="L174" s="8" t="inlineStr">
@@ -13983,7 +13983,7 @@
       </c>
       <c r="K175" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p07/p07_13_eval_and_checks.svg</t>
+          <t>docs/images/part14/p07/Yu-Project07-Fig13.svg</t>
         </is>
       </c>
       <c r="L175" s="8" t="inlineStr">
@@ -14063,7 +14063,7 @@
       </c>
       <c r="K176" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p07/p07_14_roadmap.svg</t>
+          <t>docs/images/part14/p07/Yu-Project07-Fig14.svg</t>
         </is>
       </c>
       <c r="L176" s="8" t="inlineStr">
@@ -14143,7 +14143,7 @@
       </c>
       <c r="K177" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p08/p08_01_dataops_platform_overview.svg</t>
+          <t>docs/images/part14/p08/Yu-Project08-Fig01.svg</t>
         </is>
       </c>
       <c r="L177" s="8" t="inlineStr">
@@ -14223,7 +14223,7 @@
       </c>
       <c r="K178" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p08/p08_02_four_layer_architecture.svg</t>
+          <t>docs/images/part14/p08/Yu-Project08-Fig02.svg</t>
         </is>
       </c>
       <c r="L178" s="8" t="inlineStr">
@@ -14303,7 +14303,7 @@
       </c>
       <c r="K179" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p08/p08_03_specs_to_ops_pipeline.svg</t>
+          <t>docs/images/part14/p08/Yu-Project08-Fig03.svg</t>
         </is>
       </c>
       <c r="L179" s="8" t="inlineStr">
@@ -14383,7 +14383,7 @@
       </c>
       <c r="K180" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p08/p08_04_object_model.svg</t>
+          <t>docs/images/part14/p08/Yu-Project08-Fig04.svg</t>
         </is>
       </c>
       <c r="L180" s="8" t="inlineStr">
@@ -14463,7 +14463,7 @@
       </c>
       <c r="K181" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p08/p08_05_version_lifecycle.svg</t>
+          <t>docs/images/part14/p08/Yu-Project08-Fig05.svg</t>
         </is>
       </c>
       <c r="L181" s="8" t="inlineStr">
@@ -14543,7 +14543,7 @@
       </c>
       <c r="K182" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p08/p08_06_experiment_tracking.svg</t>
+          <t>docs/images/part14/p08/Yu-Project08-Fig06.svg</t>
         </is>
       </c>
       <c r="L182" s="8" t="inlineStr">
@@ -14623,7 +14623,7 @@
       </c>
       <c r="K183" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p08/p08_07_lineage_graph.svg</t>
+          <t>docs/images/part14/p08/Yu-Project08-Fig07.svg</t>
         </is>
       </c>
       <c r="L183" s="8" t="inlineStr">
@@ -14703,7 +14703,7 @@
       </c>
       <c r="K184" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p08/p08_08_rollback_flow.svg</t>
+          <t>docs/images/part14/p08/Yu-Project08-Fig08.svg</t>
         </is>
       </c>
       <c r="L184" s="8" t="inlineStr">
@@ -14783,7 +14783,7 @@
       </c>
       <c r="K185" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p08/p08_09_observability_loop.svg</t>
+          <t>docs/images/part14/p08/Yu-Project08-Fig09.svg</t>
         </is>
       </c>
       <c r="L185" s="8" t="inlineStr">
@@ -14863,7 +14863,7 @@
       </c>
       <c r="K186" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p08/p08_10_audit_and_incident_review.svg</t>
+          <t>docs/images/part14/p08/Yu-Project08-Fig10.svg</t>
         </is>
       </c>
       <c r="L186" s="8" t="inlineStr">
@@ -14943,7 +14943,7 @@
       </c>
       <c r="K187" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p08/p08_11_validation_pipeline.svg</t>
+          <t>docs/images/part14/p08/Yu-Project08-Fig11.svg</t>
         </is>
       </c>
       <c r="L187" s="8" t="inlineStr">
@@ -15023,7 +15023,7 @@
       </c>
       <c r="K188" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p09/p09_01_privacy_pipeline_overview.svg</t>
+          <t>docs/images/part14/p09/Liu-Project09-Fig01.svg</t>
         </is>
       </c>
       <c r="L188" s="8" t="inlineStr">
@@ -15103,7 +15103,7 @@
       </c>
       <c r="K189" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p09/p09_02_roles_and_responsibilities.svg</t>
+          <t>docs/images/part14/p09/Liu-Project09-Fig02.svg</t>
         </is>
       </c>
       <c r="L189" s="8" t="inlineStr">
@@ -15179,7 +15179,7 @@
       </c>
       <c r="K190" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p09/p09_03_specs_layer.svg</t>
+          <t>docs/images/part14/p09/Liu-Project09-Fig03.svg</t>
         </is>
       </c>
       <c r="L190" s="8" t="inlineStr">
@@ -15259,7 +15259,7 @@
       </c>
       <c r="K191" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p09/p09_04_raw_records_coverage.svg</t>
+          <t>docs/images/part14/p09/Liu-Project09-Fig04.svg</t>
         </is>
       </c>
       <c r="L191" s="8" t="inlineStr">
@@ -15339,7 +15339,7 @@
       </c>
       <c r="K192" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p09/p09_05_pii_detection_distribution.svg</t>
+          <t>docs/images/part14/p09/Liu-Project09-Fig05.svg</t>
         </is>
       </c>
       <c r="L192" s="8" t="inlineStr">
@@ -15419,7 +15419,7 @@
       </c>
       <c r="K193" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p09/p09_06_classification_and_quarantine.svg</t>
+          <t>docs/images/part14/p09/Liu-Project09-Fig06.svg</t>
         </is>
       </c>
       <c r="L193" s="8" t="inlineStr">
@@ -15499,7 +15499,7 @@
       </c>
       <c r="K194" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p09/p09_07_redaction_strategies.svg</t>
+          <t>docs/images/part14/p09/Liu-Project09-Fig07.svg</t>
         </is>
       </c>
       <c r="L194" s="8" t="inlineStr">
@@ -15579,7 +15579,7 @@
       </c>
       <c r="K195" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p09/p09_08_storage_zones.svg</t>
+          <t>docs/images/part14/p09/Liu-Project09-Fig08.svg</t>
         </is>
       </c>
       <c r="L195" s="8" t="inlineStr">
@@ -15659,7 +15659,7 @@
       </c>
       <c r="K196" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p09/p09_09_alerts_and_audit.svg</t>
+          <t>docs/images/part14/p09/Liu-Project09-Fig09.svg</t>
         </is>
       </c>
       <c r="L196" s="8" t="inlineStr">
@@ -15739,7 +15739,7 @@
       </c>
       <c r="K197" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p09/p09_10_preflight_checks.svg</t>
+          <t>docs/images/part14/p09/Liu-Project09-Fig10.svg</t>
         </is>
       </c>
       <c r="L197" s="8" t="inlineStr">
@@ -15819,7 +15819,7 @@
       </c>
       <c r="K198" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p09/p09_11_incident_postmortem.svg</t>
+          <t>docs/images/part14/p09/Liu-Project09-Fig11.svg</t>
         </is>
       </c>
       <c r="L198" s="8" t="inlineStr">
@@ -15899,7 +15899,7 @@
       </c>
       <c r="K199" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p09/p09_12_execution_sequence.svg</t>
+          <t>docs/images/part14/p09/Liu-Project09-Fig12.svg</t>
         </is>
       </c>
       <c r="L199" s="8" t="inlineStr">
@@ -15979,7 +15979,7 @@
       </c>
       <c r="K200" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p10/p10_01_flywheel_overview.svg</t>
+          <t>docs/images/part14/p10/Wang-Project10-Fig01.svg</t>
         </is>
       </c>
       <c r="L200" s="8" t="inlineStr">
@@ -16059,7 +16059,7 @@
       </c>
       <c r="K201" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p10/p10_02_registry_and_interfaces.svg</t>
+          <t>docs/images/part14/p10/Wang-Project10-Fig02.svg</t>
         </is>
       </c>
       <c r="L201" s="8" t="inlineStr">
@@ -16139,7 +16139,7 @@
       </c>
       <c r="K202" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p10/p10_03_project_specs.svg</t>
+          <t>docs/images/part14/p10/Wang-Project10-Fig03.svg</t>
         </is>
       </c>
       <c r="L202" s="8" t="inlineStr">
@@ -16219,7 +16219,7 @@
       </c>
       <c r="K203" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p10/p10_04_stage_plan.svg</t>
+          <t>docs/images/part14/p10/Wang-Project10-Fig04.svg</t>
         </is>
       </c>
       <c r="L203" s="8" t="inlineStr">
@@ -16299,7 +16299,7 @@
       </c>
       <c r="K204" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p10/p10_05_architecture_code_mapping.svg</t>
+          <t>docs/images/part14/p10/Wang-Project10-Fig05.svg</t>
         </is>
       </c>
       <c r="L204" s="8" t="inlineStr">
@@ -16379,7 +16379,7 @@
       </c>
       <c r="K205" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p10/p10_06_boundaries_and_control_points.svg</t>
+          <t>docs/images/part14/p10/Wang-Project10-Fig06.svg</t>
         </is>
       </c>
       <c r="L205" s="8" t="inlineStr">
@@ -16459,7 +16459,7 @@
       </c>
       <c r="K206" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p10/p10_07_runs_and_milestones.svg</t>
+          <t>docs/images/part14/p10/Wang-Project10-Fig07.svg</t>
         </is>
       </c>
       <c r="L206" s="8" t="inlineStr">
@@ -16539,7 +16539,7 @@
       </c>
       <c r="K207" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p10/p10_08_bottleneck_map.svg</t>
+          <t>docs/images/part14/p10/Wang-Project10-Fig08.svg</t>
         </is>
       </c>
       <c r="L207" s="8" t="inlineStr">
@@ -16619,7 +16619,7 @@
       </c>
       <c r="K208" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p10/p10_09_metrics_codegen.svg</t>
+          <t>docs/images/part14/p10/Wang-Project10-Fig09.svg</t>
         </is>
       </c>
       <c r="L208" s="8" t="inlineStr">
@@ -16699,7 +16699,7 @@
       </c>
       <c r="K209" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p10/p10_10_check_contracts.svg</t>
+          <t>docs/images/part14/p10/Wang-Project10-Fig10.svg</t>
         </is>
       </c>
       <c r="L209" s="8" t="inlineStr">
@@ -16779,7 +16779,7 @@
       </c>
       <c r="K210" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p11_mini_deepseek_arch_en.svg</t>
+          <t>docs/images/part14/Yu-Project11-Fig02-EN.svg</t>
         </is>
       </c>
       <c r="L210" s="8" t="inlineStr">
@@ -16859,7 +16859,7 @@
       </c>
       <c r="K211" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p12/p12_r1_reasoning_flywheel_architecture.svg</t>
+          <t>docs/images/part14/p12/Wang-Project12-Fig01.svg</t>
         </is>
       </c>
       <c r="L211" s="8" t="inlineStr">
@@ -16937,7 +16937,7 @@
       </c>
       <c r="K212" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p13_mm_instruction_factory_arch_en.svg</t>
+          <t>docs/images/part14/Yu-Project13-Fig02-EN.svg</t>
         </is>
       </c>
       <c r="L212" s="8" t="inlineStr">
@@ -17017,7 +17017,7 @@
       </c>
       <c r="K213" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p14_video_generation_pipeline_en.svg</t>
+          <t>docs/images/part14/Luo-Project14-Fig04-EN.svg</t>
         </is>
       </c>
       <c r="L213" s="8" t="inlineStr">
@@ -17093,7 +17093,7 @@
       </c>
       <c r="K214" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p14_video_frame_0.jpg</t>
+          <t>docs/images/part14/Luo-Project14-Fig01.jpg</t>
         </is>
       </c>
       <c r="L214" s="8" t="inlineStr">
@@ -17169,7 +17169,7 @@
       </c>
       <c r="K215" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p14_video_frame_1.jpg</t>
+          <t>docs/images/part14/Luo-Project14-Fig02.jpg</t>
         </is>
       </c>
       <c r="L215" s="8" t="inlineStr">
@@ -17245,7 +17245,7 @@
       </c>
       <c r="K216" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p15_dataagent_engineering_chain_en.png</t>
+          <t>docs/images/part14/Cao-Project15-Fig03-EN.png</t>
         </is>
       </c>
       <c r="L216" s="8" t="inlineStr">
@@ -17321,7 +17321,7 @@
       </c>
       <c r="K217" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p15_datagallery_architecture_vector.svg</t>
+          <t>docs/images/part14/Cao-Project15-Fig08.svg</t>
         </is>
       </c>
       <c r="L217" s="8" t="inlineStr">
@@ -17397,7 +17397,7 @@
       </c>
       <c r="K218" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/p15_dataagent_semantic_bi_sequence_en.svg</t>
+          <t>docs/images/part14/Cao-Project15-Fig07-EN.svg</t>
         </is>
       </c>
       <c r="L218" s="8" t="inlineStr">
@@ -17471,7 +17471,7 @@
       </c>
       <c r="K219" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part2/pretrain_data_source_map.svg</t>
+          <t>docs/images/part2/Yu-Chap04-Fig01.svg</t>
         </is>
       </c>
       <c r="L219" s="8" t="inlineStr">
@@ -17545,7 +17545,7 @@
       </c>
       <c r="K220" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part2/data_ingestion_provenance_chain.svg</t>
+          <t>docs/images/part2/Yu-Chap04-Fig02.svg</t>
         </is>
       </c>
       <c r="L220" s="8" t="inlineStr">
@@ -17619,7 +17619,7 @@
       </c>
       <c r="K221" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part2/cleaning_pipeline_overview.svg</t>
+          <t>docs/images/part2/Yu-Chap05-Fig01.svg</t>
         </is>
       </c>
       <c r="L221" s="8" t="inlineStr">
@@ -17693,7 +17693,7 @@
       </c>
       <c r="K222" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part2/quality_filter_funnel_loop.svg</t>
+          <t>docs/images/part2/Yu-Chap05-Fig02.svg</t>
         </is>
       </c>
       <c r="L222" s="8" t="inlineStr">
@@ -17767,7 +17767,7 @@
       </c>
       <c r="K223" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part2/io_bottleneck_diagnosis_flow.svg</t>
+          <t>docs/images/part2/Wang-Chap06-Fig01.svg</t>
         </is>
       </c>
       <c r="L223" s="8" t="inlineStr">
@@ -17841,7 +17841,7 @@
       </c>
       <c r="K224" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part2/training_input_pipeline_layers.svg</t>
+          <t>docs/images/part2/Wang-Chap06-Fig02.svg</t>
         </is>
       </c>
       <c r="L224" s="8" t="inlineStr">
@@ -17915,7 +17915,7 @@
       </c>
       <c r="K225" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part2/data_operations_flywheel.svg</t>
+          <t>docs/images/part2/Wang-Chap07-Fig01.svg</t>
         </is>
       </c>
       <c r="L225" s="8" t="inlineStr">
@@ -17989,7 +17989,7 @@
       </c>
       <c r="K226" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part2/data_evaluation_loop.svg</t>
+          <t>docs/images/part2/Wang-Chap07-Fig02.svg</t>
         </is>
       </c>
       <c r="L226" s="8" t="inlineStr">
@@ -18063,7 +18063,7 @@
       </c>
       <c r="K227" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part3/multimodal_data_panorama.svg</t>
+          <t>docs/images/part3/Yu-Chap08-Fig01.svg</t>
         </is>
       </c>
       <c r="L227" s="8" t="inlineStr">
@@ -18137,7 +18137,7 @@
       </c>
       <c r="K228" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part3/image_semantic_alignment_flow.svg</t>
+          <t>docs/images/part3/Yu-Chap08-Fig02.svg</t>
         </is>
       </c>
       <c r="L228" s="8" t="inlineStr">
@@ -18211,7 +18211,7 @@
       </c>
       <c r="K229" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part3/anyres_dynamic_patching.svg</t>
+          <t>docs/images/part3/Yu-Chap08-Fig03.svg</t>
         </is>
       </c>
       <c r="L229" s="8" t="inlineStr">
@@ -18285,7 +18285,7 @@
       </c>
       <c r="K230" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part3/recaptioning_ocr_pipeline.svg</t>
+          <t>docs/images/part3/Yu-Chap09-Fig01.svg</t>
         </is>
       </c>
       <c r="L230" s="8" t="inlineStr">
@@ -18359,7 +18359,7 @@
       </c>
       <c r="K231" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part3/document_structure_sample.svg</t>
+          <t>docs/images/part3/Yu-Chap09-Fig02.svg</t>
         </is>
       </c>
       <c r="L231" s="8" t="inlineStr">
@@ -18433,7 +18433,7 @@
       </c>
       <c r="K232" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part3/av_sample_pipeline.svg</t>
+          <t>docs/images/part3/Wang-Chap10-Fig01.svg</t>
         </is>
       </c>
       <c r="L232" s="8" t="inlineStr">
@@ -18507,7 +18507,7 @@
       </c>
       <c r="K233" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part3/av_shot_boundary_hsv.svg</t>
+          <t>docs/images/part3/Wang-Chap10-Fig02.svg</t>
         </is>
       </c>
       <c r="L233" s="8" t="inlineStr">
@@ -18581,7 +18581,7 @@
       </c>
       <c r="K234" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part3/asr_whisperx_comparison.svg</t>
+          <t>docs/images/part3/Wang-Chap10-Fig03.svg</t>
         </is>
       </c>
       <c r="L234" s="8" t="inlineStr">
@@ -18655,7 +18655,7 @@
       </c>
       <c r="K235" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part3/av_alignment_diagram.svg</t>
+          <t>docs/images/part3/Wang-Chap10-Fig04.svg</t>
         </is>
       </c>
       <c r="L235" s="8" t="inlineStr">
@@ -18729,7 +18729,7 @@
       </c>
       <c r="K236" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part3/cross_modal_alignment_hierarchy.svg</t>
+          <t>docs/images/part3/Wang-Chap11-Fig01.svg</t>
         </is>
       </c>
       <c r="L236" s="8" t="inlineStr">
@@ -18803,7 +18803,7 @@
       </c>
       <c r="K237" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part3/fusion_training_sample_design.svg</t>
+          <t>docs/images/part3/Wang-Chap11-Fig02.svg</t>
         </is>
       </c>
       <c r="L237" s="8" t="inlineStr">
@@ -18877,7 +18877,7 @@
       </c>
       <c r="K238" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part4/图12_1.svg</t>
+          <t>docs/images/part4/Yu-Chap12-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L238" s="8" t="inlineStr">
@@ -18951,7 +18951,7 @@
       </c>
       <c r="K239" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part4/图12_2.svg</t>
+          <t>docs/images/part4/Yu-Chap12-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L239" s="8" t="inlineStr">
@@ -19025,7 +19025,7 @@
       </c>
       <c r="K240" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part4/图13_1.svg</t>
+          <t>docs/images/part4/Yu-Chap13-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L240" s="8" t="inlineStr">
@@ -19099,7 +19099,7 @@
       </c>
       <c r="K241" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part4/图13_2.svg</t>
+          <t>docs/images/part4/Yu-Chap13-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L241" s="8" t="inlineStr">
@@ -19173,7 +19173,7 @@
       </c>
       <c r="K242" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part4/图14_1.svg</t>
+          <t>docs/images/part4/Zhang-Chap14-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L242" s="8" t="inlineStr">
@@ -19247,7 +19247,7 @@
       </c>
       <c r="K243" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part4/图14_2.svg</t>
+          <t>docs/images/part4/Zhang-Chap14-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L243" s="8" t="inlineStr">
@@ -19321,7 +19321,7 @@
       </c>
       <c r="K244" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part5/图15_1.svg</t>
+          <t>docs/images/part5/Wang-Chap15-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L244" s="8" t="inlineStr">
@@ -19395,7 +19395,7 @@
       </c>
       <c r="K245" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part5/图15_2.svg</t>
+          <t>docs/images/part5/Wang-Chap15-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L245" s="8" t="inlineStr">
@@ -19469,7 +19469,7 @@
       </c>
       <c r="K246" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part5/图16_1.svg</t>
+          <t>docs/images/part5/Wang-Chap16-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L246" s="8" t="inlineStr">
@@ -19543,7 +19543,7 @@
       </c>
       <c r="K247" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part5/图16_2.svg</t>
+          <t>docs/images/part5/Wang-Chap16-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L247" s="8" t="inlineStr">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="K248" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part5/图17_1.svg</t>
+          <t>docs/images/part5/Zhang-Chap17-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L248" s="8" t="inlineStr">
@@ -19691,7 +19691,7 @@
       </c>
       <c r="K249" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part5/图17_2.svg</t>
+          <t>docs/images/part5/Zhang-Chap17-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L249" s="8" t="inlineStr">
@@ -19765,7 +19765,7 @@
       </c>
       <c r="K250" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part6/图18_1.svg</t>
+          <t>docs/images/part6/Yu-Chap18-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L250" s="8" t="inlineStr">
@@ -19839,7 +19839,7 @@
       </c>
       <c r="K251" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part6/图18_2.svg</t>
+          <t>docs/images/part6/Yu-Chap18-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L251" s="8" t="inlineStr">
@@ -19913,7 +19913,7 @@
       </c>
       <c r="K252" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part6/图19_1.svg</t>
+          <t>docs/images/part6/Yu-Chap19-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L252" s="8" t="inlineStr">
@@ -19987,7 +19987,7 @@
       </c>
       <c r="K253" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part6/图19_2.svg</t>
+          <t>docs/images/part6/Yu-Chap19-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L253" s="8" t="inlineStr">
@@ -20061,7 +20061,7 @@
       </c>
       <c r="K254" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part6/图20_1.svg</t>
+          <t>docs/images/part6/Zhang-Chap20-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L254" s="8" t="inlineStr">
@@ -20135,7 +20135,7 @@
       </c>
       <c r="K255" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part6/图20_2.svg</t>
+          <t>docs/images/part6/Zhang-Chap20-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L255" s="8" t="inlineStr">
@@ -20209,7 +20209,7 @@
       </c>
       <c r="K256" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图21_1.svg</t>
+          <t>docs/images/part7/Du-Chap21-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L256" s="8" t="inlineStr">
@@ -20283,7 +20283,7 @@
       </c>
       <c r="K257" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图21_2.svg</t>
+          <t>docs/images/part7/Du-Chap21-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L257" s="8" t="inlineStr">
@@ -20357,7 +20357,7 @@
       </c>
       <c r="K258" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图21_3.svg</t>
+          <t>docs/images/part7/Du-Chap21-Fig03-ZH.svg</t>
         </is>
       </c>
       <c r="L258" s="8" t="inlineStr">
@@ -20431,7 +20431,7 @@
       </c>
       <c r="K259" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图21_4.svg</t>
+          <t>docs/images/part7/Du-Chap21-Fig04-ZH.svg</t>
         </is>
       </c>
       <c r="L259" s="8" t="inlineStr">
@@ -20505,7 +20505,7 @@
       </c>
       <c r="K260" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图21_5.svg</t>
+          <t>docs/images/part7/Du-Chap21-Fig05-ZH.svg</t>
         </is>
       </c>
       <c r="L260" s="8" t="inlineStr">
@@ -20579,7 +20579,7 @@
       </c>
       <c r="K261" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图21_6.svg</t>
+          <t>docs/images/part7/Du-Chap21-Fig06-ZH.svg</t>
         </is>
       </c>
       <c r="L261" s="8" t="inlineStr">
@@ -20653,7 +20653,7 @@
       </c>
       <c r="K262" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图21_7.svg</t>
+          <t>docs/images/part7/Du-Chap21-Fig07-ZH.svg</t>
         </is>
       </c>
       <c r="L262" s="8" t="inlineStr">
@@ -20727,7 +20727,7 @@
       </c>
       <c r="K263" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图21_8.svg</t>
+          <t>docs/images/part7/Du-Chap21-Fig08-ZH.svg</t>
         </is>
       </c>
       <c r="L263" s="8" t="inlineStr">
@@ -20801,7 +20801,7 @@
       </c>
       <c r="K264" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图21_9.svg</t>
+          <t>docs/images/part7/Du-Chap21-Fig09-ZH.svg</t>
         </is>
       </c>
       <c r="L264" s="8" t="inlineStr">
@@ -20875,7 +20875,7 @@
       </c>
       <c r="K265" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图22_1.svg</t>
+          <t>docs/images/part7/Du-Chap22-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L265" s="8" t="inlineStr">
@@ -20949,7 +20949,7 @@
       </c>
       <c r="K266" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图22_2.svg</t>
+          <t>docs/images/part7/Du-Chap22-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L266" s="8" t="inlineStr">
@@ -21023,7 +21023,7 @@
       </c>
       <c r="K267" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图22_3.svg</t>
+          <t>docs/images/part7/Du-Chap22-Fig03-ZH.svg</t>
         </is>
       </c>
       <c r="L267" s="8" t="inlineStr">
@@ -21097,7 +21097,7 @@
       </c>
       <c r="K268" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图22_4.svg</t>
+          <t>docs/images/part7/Du-Chap22-Fig04-ZH.svg</t>
         </is>
       </c>
       <c r="L268" s="8" t="inlineStr">
@@ -21171,7 +21171,7 @@
       </c>
       <c r="K269" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图22_5.svg</t>
+          <t>docs/images/part7/Du-Chap22-Fig05-ZH.svg</t>
         </is>
       </c>
       <c r="L269" s="8" t="inlineStr">
@@ -21245,7 +21245,7 @@
       </c>
       <c r="K270" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图23_1.svg</t>
+          <t>docs/images/part7/Yu-Chap23-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L270" s="8" t="inlineStr">
@@ -21319,7 +21319,7 @@
       </c>
       <c r="K271" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图23_2.svg</t>
+          <t>docs/images/part7/Yu-Chap23-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L271" s="8" t="inlineStr">
@@ -21393,7 +21393,7 @@
       </c>
       <c r="K272" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图23_3.svg</t>
+          <t>docs/images/part7/Yu-Chap23-Fig03-ZH.svg</t>
         </is>
       </c>
       <c r="L272" s="8" t="inlineStr">
@@ -21467,7 +21467,7 @@
       </c>
       <c r="K273" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part7/图23_4.svg</t>
+          <t>docs/images/part7/Yu-Chap23-Fig04-ZH.svg</t>
         </is>
       </c>
       <c r="L273" s="8" t="inlineStr">
@@ -21541,7 +21541,7 @@
       </c>
       <c r="K274" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part8/图24_1.svg</t>
+          <t>docs/images/part8/Yu-Chap24-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L274" s="8" t="inlineStr">
@@ -21615,7 +21615,7 @@
       </c>
       <c r="K275" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part8/图24_2.svg</t>
+          <t>docs/images/part8/Yu-Chap24-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L275" s="8" t="inlineStr">
@@ -21693,7 +21693,7 @@
       </c>
       <c r="K276" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part8/图24_3.svg</t>
+          <t>docs/images/part8/Yu-Chap24-Fig03-ZH.svg</t>
         </is>
       </c>
       <c r="L276" s="8" t="inlineStr">
@@ -21771,7 +21771,7 @@
       </c>
       <c r="K277" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part8/图25_1.svg</t>
+          <t>docs/images/part8/Du-Chap25-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L277" s="8" t="inlineStr">
@@ -21849,7 +21849,7 @@
       </c>
       <c r="K278" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part8/图25_2.svg</t>
+          <t>docs/images/part8/Du-Chap25-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L278" s="8" t="inlineStr">
@@ -21927,7 +21927,7 @@
       </c>
       <c r="K279" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part8/图26_1.svg</t>
+          <t>docs/images/part8/Du-Chap26-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L279" s="8" t="inlineStr">
@@ -22005,7 +22005,7 @@
       </c>
       <c r="K280" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part8/图26_2.svg</t>
+          <t>docs/images/part8/Du-Chap26-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L280" s="8" t="inlineStr">
@@ -22083,7 +22083,7 @@
       </c>
       <c r="K281" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part9/图27_1.svg</t>
+          <t>docs/images/part9/Zhang-Chap27-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L281" s="8" t="inlineStr">
@@ -22157,7 +22157,7 @@
       </c>
       <c r="K282" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part9/图27_2.svg</t>
+          <t>docs/images/part9/Zhang-Chap27-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L282" s="8" t="inlineStr">
@@ -22231,7 +22231,7 @@
       </c>
       <c r="K283" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part9/图27_3.svg</t>
+          <t>docs/images/part9/Zhang-Chap27-Fig03-ZH.svg</t>
         </is>
       </c>
       <c r="L283" s="8" t="inlineStr">
@@ -22305,7 +22305,7 @@
       </c>
       <c r="K284" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part9/图27_4.svg</t>
+          <t>docs/images/part9/Zhang-Chap27-Fig04-ZH.svg</t>
         </is>
       </c>
       <c r="L284" s="8" t="inlineStr">
@@ -22379,7 +22379,7 @@
       </c>
       <c r="K285" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part9/图28_1.svg</t>
+          <t>docs/images/part9/Liu-Chap28-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L285" s="8" t="inlineStr">
@@ -22453,7 +22453,7 @@
       </c>
       <c r="K286" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part9/图28_2.svg</t>
+          <t>docs/images/part9/Liu-Chap28-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L286" s="8" t="inlineStr">
@@ -22531,7 +22531,7 @@
       </c>
       <c r="K287" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part9/图28_3.svg</t>
+          <t>docs/images/part9/Liu-Chap28-Fig03-ZH.svg</t>
         </is>
       </c>
       <c r="L287" s="8" t="inlineStr">
@@ -22605,7 +22605,7 @@
       </c>
       <c r="K288" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part9/图28_4.svg</t>
+          <t>docs/images/part9/Liu-Chap28-Fig04-ZH.svg</t>
         </is>
       </c>
       <c r="L288" s="8" t="inlineStr">
@@ -22679,7 +22679,7 @@
       </c>
       <c r="K289" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part9/图29_1.svg</t>
+          <t>docs/images/part9/Liu-Chap29-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L289" s="8" t="inlineStr">
@@ -22753,7 +22753,7 @@
       </c>
       <c r="K290" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part9/图29_2.svg</t>
+          <t>docs/images/part9/Liu-Chap29-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L290" s="8" t="inlineStr">
@@ -22827,7 +22827,7 @@
       </c>
       <c r="K291" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part9/图29_3.svg</t>
+          <t>docs/images/part9/Liu-Chap29-Fig03-ZH.svg</t>
         </is>
       </c>
       <c r="L291" s="8" t="inlineStr">
@@ -22905,7 +22905,7 @@
       </c>
       <c r="K292" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part9/图30_1.svg</t>
+          <t>docs/images/part9/Luo-Chap30-Fig01-ZH.svg</t>
         </is>
       </c>
       <c r="L292" s="8" t="inlineStr">
@@ -22979,7 +22979,7 @@
       </c>
       <c r="K293" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part9/图30_2.svg</t>
+          <t>docs/images/part9/Luo-Chap30-Fig02-ZH.svg</t>
         </is>
       </c>
       <c r="L293" s="8" t="inlineStr">

</xml_diff>